<commit_message>
feat(gate): Chicago-time sessions, session field rename, and funded payout rules
- Session/break anchored to America/Chicago; fix CME break to 16:00-17:00 CT
- Logs and audit timestamps in configurable zone (default America/Chicago) instead of UTC
- Rename session_start_time_et/session_flatten_time_et to session_start_time/session_flatten_time (CT values)
- Funded: add buffer, payout, derived balance_for_payout; trailing floor capped at min_account_balance
- Funded day lock only after balance_for_payout is reached; payout status validates against it
- Deterministic tests (fixed dates) and Rules/Lucid.xlsx payout data
</commit_message>
<xml_diff>
--- a/Rules/Lucid.xlsx
+++ b/Rules/Lucid.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/albertocordero/Documents/PI/Claude-Trading/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/albertocordero/Documents/PI/Claude-Trading/Rules/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{865D8B2E-D0FD-F940-833E-783DE9295287}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85917353-1564-A942-BEC7-A42C0A48AA51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{28763908-CE87-F442-A76F-9B45EB43C639}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="32">
   <si>
     <t>25K FLEX FUNDED</t>
   </si>
@@ -117,6 +117,24 @@
   </si>
   <si>
     <t>Minimum Balance</t>
+  </si>
+  <si>
+    <t>Buffer</t>
+  </si>
+  <si>
+    <t>Payout</t>
+  </si>
+  <si>
+    <t>25K FLEX PAYOUT</t>
+  </si>
+  <si>
+    <t>50K FLEX PAYOUT</t>
+  </si>
+  <si>
+    <t>100K FLEX PAYOUT</t>
+  </si>
+  <si>
+    <t>Balance for Payout</t>
   </si>
 </sst>
 </file>
@@ -125,10 +143,10 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="44" formatCode="_(&quot;₡&quot;* #,##0.00_);_(&quot;₡&quot;* \(#,##0.00\);_(&quot;₡&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="166" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="168" formatCode="_([$$-409]* #,##0_);_([$$-409]* \(#,##0\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="164" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_([$$-409]* #,##0_);_([$$-409]* \(#,##0\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -139,6 +157,12 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -165,18 +189,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -512,14 +539,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10646601-8FE2-6C4B-9B3C-9C985AD108E2}">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="7" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="10" width="17.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="B1" t="s">
         <v>17</v>
       </c>
@@ -538,8 +565,17 @@
       <c r="G1" s="1" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>18</v>
       </c>
@@ -561,8 +597,17 @@
       <c r="G2" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>19</v>
       </c>
@@ -584,8 +629,17 @@
       <c r="G3" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>1</v>
       </c>
@@ -607,8 +661,17 @@
       <c r="G4" s="2">
         <v>3000</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H4" s="2">
+        <v>1000</v>
+      </c>
+      <c r="I4" s="2">
+        <v>2000</v>
+      </c>
+      <c r="J4" s="2">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>2</v>
       </c>
@@ -630,8 +693,17 @@
       <c r="G5" s="2">
         <v>1800</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H5" s="2">
+        <v>600</v>
+      </c>
+      <c r="I5" s="2">
+        <v>1200</v>
+      </c>
+      <c r="J5" s="2">
+        <v>1800</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -653,8 +725,17 @@
       <c r="G6" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -676,8 +757,17 @@
       <c r="G7" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -699,8 +789,17 @@
       <c r="G8" s="1" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -722,8 +821,17 @@
       <c r="G9" s="1" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>6</v>
       </c>
@@ -745,8 +853,17 @@
       <c r="G10" s="1">
         <v>5</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H10" s="1">
+        <v>5</v>
+      </c>
+      <c r="I10" s="1">
+        <v>5</v>
+      </c>
+      <c r="J10" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -768,8 +885,17 @@
       <c r="G11" s="1" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="H11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -791,38 +917,161 @@
       <c r="G12" s="4">
         <v>100100</v>
       </c>
-    </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B17" s="2"/>
+      <c r="H12" s="4">
+        <v>25100</v>
+      </c>
+      <c r="I12" s="4">
+        <v>50100</v>
+      </c>
+      <c r="J12" s="4">
+        <v>100100</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E13" s="4">
+        <v>27100</v>
+      </c>
+      <c r="F13" s="4">
+        <v>54100</v>
+      </c>
+      <c r="G13" s="4">
+        <v>106100</v>
+      </c>
+      <c r="H13" s="4">
+        <v>28100</v>
+      </c>
+      <c r="I13" s="4">
+        <v>56100</v>
+      </c>
+      <c r="J13" s="4">
+        <v>109100</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14">
+        <v>1100</v>
+      </c>
+      <c r="F14">
+        <v>2100</v>
+      </c>
+      <c r="G14">
+        <v>3100</v>
+      </c>
+      <c r="H14">
+        <v>1100</v>
+      </c>
+      <c r="I14">
+        <v>2100</v>
+      </c>
+      <c r="J14">
+        <v>3100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>27</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1000</v>
+      </c>
+      <c r="F15" s="1">
+        <v>2000</v>
+      </c>
+      <c r="G15" s="1">
+        <v>3000</v>
+      </c>
+      <c r="H15" s="1">
+        <v>2000</v>
+      </c>
+      <c r="I15" s="1">
+        <v>4000</v>
+      </c>
+      <c r="J15" s="1">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="B16" s="1"/>
+      <c r="C16" s="1"/>
+      <c r="D16" s="1"/>
+      <c r="E16" s="5"/>
+      <c r="F16" s="5"/>
+      <c r="G16" s="5"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
+      <c r="J16" s="5"/>
+    </row>
+    <row r="17" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B18" s="2"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+    </row>
+    <row r="18" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.2">
+      <c r="E18" s="1"/>
+      <c r="F18" s="1"/>
+      <c r="G18" s="1"/>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B19" s="2"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>